<commit_message>
docs: simplifica modelo de planilha de comparativo
</commit_message>
<xml_diff>
--- a/public/modelo_comparativo.xlsx
+++ b/public/modelo_comparativo.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Acumulado" sheetId="1" r:id="rId1"/>
+    <sheet name="Modelo_Acumulado" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,11 +397,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>NÚMERO DOCUMENTO</v>
+        <v>ROMANEIO</v>
       </c>
       <c r="B1" t="str">
         <v>PRODUTOR</v>
@@ -413,75 +413,29 @@
         <v>PESO LÍQUIDO C/ DESCONTO (KG)</v>
       </c>
       <c r="E1" t="str">
-        <v>TESTE</v>
-      </c>
-      <c r="F1" t="str">
-        <v>UNIDADE</v>
+        <v>RESULTADO DO TESTE</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>252</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>VICENTE RIVA</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>ITN3683</v>
-      </c>
-      <c r="D2">
-        <v>13910</v>
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>Declarada</v>
-      </c>
-      <c r="F2" t="str">
-        <v>UNIDADE EXEMPLO</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>253</v>
-      </c>
-      <c r="B3" t="str">
-        <v>EXEMPLO RATEIO 1</v>
-      </c>
-      <c r="C3" t="str">
-        <v>ABC1234</v>
-      </c>
-      <c r="D3">
-        <v>5000</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Negativa</v>
-      </c>
-      <c r="F3" t="str">
-        <v>UNIDADE EXEMPLO</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>253</v>
-      </c>
-      <c r="B4" t="str">
-        <v>EXEMPLO RATEIO 2</v>
-      </c>
-      <c r="C4" t="str">
-        <v>ABC1234</v>
-      </c>
-      <c r="D4">
-        <v>8000</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Negativa</v>
-      </c>
-      <c r="F4" t="str">
-        <v>UNIDADE EXEMPLO</v>
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>